<commit_message>
style(docs): format and align dulieubaibao.xlsx with professional styles, column widths, and zebra striping
</commit_message>
<xml_diff>
--- a/docs/dulieubaibao.xlsx
+++ b/docs/dulieubaibao.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -44,8 +44,37 @@
       <charset val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00002060"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,8 +87,32 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5F9"/>
+        <bgColor rgb="00F2F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -82,11 +135,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="medium">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="0016365C"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="0016365C"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -94,6 +189,43 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -354,399 +486,377 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>DANH SÁCH DATASET - Phát hiện tin giả bằng LLM</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="5" t="n"/>
+    </row>
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Tên dataset</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Ngôn ngữ</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Domain / Nguồn</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Quy mô (số mẫu)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Nhãn / Label</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Ngày cập nhật</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>Đánh giá / Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="75" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>High-Will/ViWikiFC</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/High-Will/ViWikiFC</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Vietnamese</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Wikipedia tiếng Việt (Fact-Checking / Bách khoa toàn thư)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>20,919 mẫu (Train: 16,738 | Dev: 2,090 | Test: 2,091)</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>3 nhãn chuẩn FEVER: SUPPORTS (Đúng/Hỗ trợ), REFUTES (Sai/Bác bỏ), NOT ENOUGH INFO (Không đủ thông tin)</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>2024 (arXiv:2405.07615)</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="11" t="inlineStr">
         <is>
           <t>Tập dữ liệu kiểm chứng thông tin (Fact Verification) dựa trên ngữ cảnh Wikipedia. Trong hệ thống phát hiện tin giả bằng LLM, đóng vai trò là module đối soát sự thật (Fact-checking Verification / RAG) nhằm xác minh xem một luận điểm cụ thể có bằng chứng xác thực hay không.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>ReliableAI/ReINTEL (VLSP 2020)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/ReliableAI/ReINTEL</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Vietnamese</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Mạng xã hội tiếng Việt (Facebook, tin tức lan truyền mạng xã hội)</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>~8,000 – 10,000 bài đăng (Train: 5,998 | Test: 2,000)</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>2 nhãn nhị phân: 0 - Reliable (Tin thật, đáng tin cậy) | 1 - Unreliable (Tin giả, tin đồn thất thiệt, sai sự thật)</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>2020 – 2021 (VLSP Shared Task)</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>Benchmark chuẩn quốc gia của Việt Nam chuyên biệt cho bài toán Phát hiện tin giả trên mạng xã hội. Khác với kiểm tra đúng sai đơn thuần, bài đăng chứa ngôn ngữ đời sống, clickbait, ngữ cảnh mạng xã hội; rất thích hợp để fine-tune hoặc đánh giá năng lực phân loại tin giả của các LLM tiếng Việt (PhoBERT, ViT5, Vistral, LLaMA-3-Vietnamese).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="85" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>tranthaihoa/ViFactCheck (AAAI 2025)</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/tranthaihoa/vifactcheck</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Vietnamese</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Báo chí điện tử chính thống đa lĩnh vực (9 đầu báo uy tín Việt Nam, 12 chủ đề: thời sự, y tế, kinh tế, xã hội...)</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t>7,232 cặp claim - evidence kèm toàn văn bài báo (full article context)</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>3 nhãn: Supported (Tin thật/Được chứng thực), Refuted (Tin giả/Bị bác bỏ), Not Enough Information (Chưa đủ thông tin)</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>2024 – 2025 (Công bố tại AAAI-25)</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="11" t="inlineStr">
         <is>
           <t>Cầu nối trực tiếp giữa bài báo tin tức (News Article) và kiểm chứng sự thật. Khắc phục nhược điểm của Wikipedia bằng cách lấy tin tức thời sự thực tế từ báo chí, giúp LLM vừa phân tích ngữ cảnh toàn bài báo vừa trích xuất bằng chứng để phát hiện tin tức bị làm giả hoặc xuyên tạc.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>WhySchools/VFND (Vietnamese Fake News Dataset)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>https://github.com/WhySchools/VFND-vietnamese-fake-news-datasets</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Vietnamese</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Các trang tin tức, báo mạng trực tuyến tiếng Việt (báo chính thống vs trang tin rác, tin đồn)</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>223 bài báo nguyên văn đầy đủ (127 tin thật, 96 tin giả)</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>2 nhãn nhị phân: Real (Tin thật) | Fake (Tin giả)</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="16" t="inlineStr">
         <is>
           <t>Bộ dữ liệu phân loại tin giả cấp bài báo hoàn chỉnh (Full-length news articles). Cực kỳ phù hợp cho hướng tiếp cận phân tích văn phong (Stylometric analysis), phát hiện ngữ điệu giật gân, câu view hoặc ngụy tạo thông tin bằng LLM thông qua kỹ thuật Prompting (Zero-shot / Chain-of-Thought).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>GonzaloA/fake_news (ISOT Fake News Benchmark)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/GonzaloA/fake_news</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>English (Đối chuẩn quốc tế)</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Tin tức thế giới thực tế từ Reuters (tin thật) và các website tin giả/chính trị không xác thực</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>44,898 bài báo đầy đủ (Train: 24,353 | Validation: 6,089 | Test: 14,456)</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>2 nhãn nhị phân: 0 - Fake (Tin giả) | 1 - Real (Tin thật)</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>2022 – 2024 (Phiên bản Hugging Face)</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="11" t="inlineStr">
         <is>
           <t>Benchmark phát hiện tin tức giả quy mô lớn nổi tiếng thế giới. Cần thiết để nhóm so sánh và đánh giá năng lực nhận biết tin giả của các nền tảng LLM lớn (GPT-4, LLaMA-3, Mistral, Qwen-2.5) trước khi thử nghiệm hoặc transfer learning về dữ liệu tiếng Việt.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="9" ht="85" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>ucsbnlp/liar (LIAR Benchmark)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>https://huggingface.co/datasets/ucsbnlp/liar</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Phát ngôn chính trị và tin tức truyền thông từ tổ chức kiểm chứng PolitiFact</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>12,836 phát biểu kèm ngữ cảnh, người nói, nguồn gốc</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>6 mức độ xác thực chi tiết: pants-fire (hoàn toàn bịa đặt), false (sai), barely-true (gần như sai), half-true (đúng một nửa), mostly-true (phần lớn đúng), true (đúng sự thật)</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>ACL Benchmark (Hugging Face)</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>Dataset tiêu chuẩn vàng cho bài toán phát hiện tin giả nhiều mức độ. Thích hợp để huấn luyện LLM giải thích lý do vì sao một thông tin bị coi là giả (Explainable Fake News Detection) thay vì chỉ phân loại nhị phân 0/1.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-    </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -761,61 +871,69 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>DANH SÁCH MÔ HÌNH / PAPER ĐỀ XUẤT - Phát hiện tin giả bằng LLM</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="31.5" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="5" t="n"/>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="5" t="n"/>
+    </row>
+    <row r="2" ht="12" customHeight="1"/>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Tên paper/mô hình</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Năm</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Kỹ thuật chính</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Kết quả nổi bật (Accuracy/F1)</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Áp dụng cho tác vụ nào</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Ngày cập nhật</t>
         </is>
@@ -826,54 +944,54 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="10" t="n"/>
       <c r="I4" s="3" t="n"/>
     </row>
-    <row r="5" ht="50" customHeight="1">
-      <c r="A5" s="3" t="n">
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>SemViQA</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2503.00955</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Semantic Evidence Retrieval (SER) + Two-step Verdict Classification (TVC)</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>80.82% strict acc trên ViWikiFC, 78.97% trên ISE-DSC01; bản Faster nhanh hơn 7x</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>Fact verification tiếng Việt (SOTA)</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
@@ -884,88 +1002,91 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="11" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="11" t="n"/>
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="10" t="n"/>
       <c r="I6" s="3" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="15" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="15" t="n"/>
       <c r="I7" s="3" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="10" t="n"/>
       <c r="I8" s="3" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="16" t="n"/>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="15" t="n"/>
       <c r="I9" s="3" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="n">
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="3" t="n"/>
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="10" t="n"/>
       <c r="I10" s="3" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="n">
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="16" t="n"/>
+      <c r="H11" s="15" t="n"/>
       <c r="I11" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add comprehensive report section for Vo Bach Kim Thinh and update surveyed baselines in dulieubaibao.xlsx
</commit_message>
<xml_diff>
--- a/docs/dulieubaibao.xlsx
+++ b/docs/dulieubaibao.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -73,6 +73,16 @@
       <color rgb="00000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -112,7 +122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -177,11 +187,69 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -226,6 +294,26 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -506,14 +594,14 @@
           <t>DANH SÁCH DATASET - Phát hiện tin giả bằng LLM</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-      <c r="C1" s="5" t="n"/>
-      <c r="D1" s="5" t="n"/>
-      <c r="E1" s="5" t="n"/>
-      <c r="F1" s="5" t="n"/>
-      <c r="G1" s="5" t="n"/>
-      <c r="H1" s="5" t="n"/>
-      <c r="I1" s="5" t="n"/>
+      <c r="B1" s="17" t="n"/>
+      <c r="C1" s="17" t="n"/>
+      <c r="D1" s="17" t="n"/>
+      <c r="E1" s="17" t="n"/>
+      <c r="F1" s="17" t="n"/>
+      <c r="G1" s="17" t="n"/>
+      <c r="H1" s="17" t="n"/>
+      <c r="I1" s="18" t="n"/>
     </row>
     <row r="2" ht="12" customHeight="1"/>
     <row r="3" ht="30" customHeight="1">
@@ -868,7 +956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -888,13 +976,14 @@
           <t>DANH SÁCH MÔ HÌNH / PAPER ĐỀ XUẤT - Phát hiện tin giả bằng LLM</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-      <c r="C1" s="5" t="n"/>
-      <c r="D1" s="5" t="n"/>
-      <c r="E1" s="5" t="n"/>
-      <c r="F1" s="5" t="n"/>
-      <c r="G1" s="5" t="n"/>
-      <c r="H1" s="5" t="n"/>
+      <c r="B1" s="17" t="n"/>
+      <c r="C1" s="17" t="n"/>
+      <c r="D1" s="17" t="n"/>
+      <c r="E1" s="17" t="n"/>
+      <c r="F1" s="17" t="n"/>
+      <c r="G1" s="17" t="n"/>
+      <c r="H1" s="17" t="n"/>
+      <c r="I1" s="18" t="n"/>
     </row>
     <row r="2" ht="12" customHeight="1"/>
     <row r="3" ht="30" customHeight="1">
@@ -944,102 +1033,230 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="n">
+    <row r="4" ht="65" customHeight="1">
+      <c r="A4" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="11" t="n"/>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="11" t="n"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="3" t="n"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="15" t="n">
+      <c r="B4" s="20" t="inlineStr">
+        <is>
+          <t>ViWikiFC Baseline (BM25 + InfoXLM-Large)</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2405.07615</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>BM25 cho Evidence Retrieval + InfoXLM-Large (Cross-Encoder) cho Verdict Prediction 3 nhãn</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>ER Acc: 88.30% (Supports), 86.93% (Refutes), 56.67% (NEI); VP F1: 86.51%; Strict Acc toàn pipeline: 67.00%</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Fact-checking tiếng Việt (Wikipedia)</t>
+        </is>
+      </c>
+      <c r="H4" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>Baseline chính thức đầu tiên trên ViWikiFC do nhóm tác giả dataset công bố; mốc tham chiếu bắt buộc để chứng minh sự cải tiến.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1">
+      <c r="A5" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>SemViQA</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>SemViQA / SemViQA Faster (SOTA ViWikiFC)</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>https://arxiv.org/abs/2503.00955</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
-        <is>
-          <t>Semantic Evidence Retrieval (SER) + Two-step Verdict Classification (TVC)</t>
-        </is>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Semantic Evidence Retrieval (TF-IDF + QATC) + Two-step Verdict Classification (TVC: Sufficiency -&gt; Stance)</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
         <is>
           <t>80.82% strict acc trên ViWikiFC, 78.97% trên ISE-DSC01; bản Faster nhanh hơn 7x</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="G5" s="23" t="inlineStr">
         <is>
           <t>Fact verification tiếng Việt (SOTA)</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>SOTA hiện tại trên ViWikiFC, đạt giải nhất UIT Data Science Challenge - đáng làm điểm so sánh chính; chưa dùng LLM sinh (GPT/Llama)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="n">
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>SOTA hiện tại trên ViWikiFC, đạt giải nhất UIT Data Science Challenge; cảm hứng trực tiếp cho cơ chế TVC của nhóm; chưa dùng LLM sinh lời giải thích.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1">
+      <c r="A6" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="11" t="n"/>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="11" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="3" t="n"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="15" t="n">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>ViFactCheck Baseline (PhoBERT &amp; XLM-RoBERTa)</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2412.15308</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Fine-tuning Pre-trained Encoders: PhoBERT-large (đơn ngữ tiếng Việt) và XLM-RoBERTa-large (đa ngữ)</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>XLM-R Large Acc: 78.40%; Macro-F1 tốt nhất toàn bộ bài báo: 89.90% trên 12 chủ đề báo chí</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Kiểm chứng tin tức báo chí đa lĩnh vực (News Fact-Checking)</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>Baseline công bố tại AAAI 2025 trên tập báo chí chính thống Việt Nam; mốc so sánh năng lực xử lý tin tức thời sự đời thực.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="65" customHeight="1">
+      <c r="A7" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="n">
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>LLM Direct Prompting (Zero-shot / Few-shot)</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Khảo sát thực nghiệm LLM</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Direct Inference không dùng RAG: Đưa Claim trực tiếp vào LLM (Qwen2.5 / LLaMA-3 / GPT) suy luận dựa trên tri thức tiềm ẩn</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Acc &lt; 55%; Macro-F1 thấp; nhãn NEI sụt giảm nghiêm trọng; dễ bị ảo giác (hallucination) trên tin mới</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Phát hiện tin giả &amp; Kiểm chứng thông tin</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>Baseline kiểm chứng thành phần (Ablation Study) bắt buộc trong NCKH để chứng minh vai trò tất yếu của cơ chế RAG và TVC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="65" customHeight="1">
+      <c r="A8" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="3" t="n"/>
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>SER + TVC + RAG (Mô hình nhóm đề xuất)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Repository viet-factcheck</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>SER: BM25 + BGE-M3 + RRF (k=60) + BGE-Reranker-v2-m3; TVC: Sufficiency Filter -&gt; Stance; LLM Qwen2.5-7B CoT Rationale</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>Kỳ vọng Strict Acc &gt; 82%, Macro-F1 &gt; 90%; Sinh lời giải thích tiếng Việt định dạng JSON có cấu trúc Pydantic</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Kiểm chứng tin tức &amp; Sinh giải thích minh bạch (Explainable Fact-Checking)</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I8" s="20" t="inlineStr">
+        <is>
+          <t>Mô hình đề xuất chính của đề tài; kết hợp thế mạnh của truy xuất ngữ nghĩa lai ghép, phân loại 2 tầng giải quyết lệch nhãn NEI và LLM sinh lời giải thích.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="40" customHeight="1">
       <c r="A9" s="15" t="n">
@@ -1080,12 +1297,17 @@
       <c r="H11" s="15" t="n"/>
       <c r="I11" s="3" t="n"/>
     </row>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>